<commit_message>
Raise the Calibre Verdict fee to USD 6,000
Rate card, service definition, time log, READMEs and the decisions log now
carry USD 6,000 with the 50/50 terms unchanged. At the USD 350 hurdle the
fee buys 17.1 all-in hours against the 15.75-hour budget. The market
rationale (product/PRICING.md) follows in the next commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BTLr4iYcvkGMcb7AZEM3uQ
</commit_message>
<xml_diff>
--- a/kit/Calibre_Engagement_Time_Log.xlsx
+++ b/kit/Calibre_Engagement_Time_Log.xlsx
@@ -94,7 +94,7 @@
     <t xml:space="preserve">Calibre Verdict fee (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Rate card, founder decision 30 Sep 2026. Not a market benchmark.</t>
+    <t xml:space="preserve">Rate card, founder decision 5 Oct 2026. Rationale in product/PRICING.md.</t>
   </si>
   <si>
     <t xml:space="preserve">Management hour cap (all-in)</t>
@@ -989,7 +989,7 @@
         <v>22</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>5500</v>
+        <v>6000</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>23</v>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">IF(OR(N(C6)=0,N(C7)=0),"",C7/C6)</f>
-        <v>15.7142857142857</v>
+        <v>17.1428571428571</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>30</v>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C15" s="13" t="n">
         <f aca="false">IF(C12="","",C12-C14)</f>
-        <v>-0.0357142857142865</v>
+        <v>1.39285714285714</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>36</v>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="C38" s="22" t="n">
         <f aca="false">IF(N(C37)=0,"",Assumptions!$C$7/C37)</f>
-        <v>349.206349206349</v>
+        <v>380.952380952381</v>
       </c>
       <c r="D38" s="22" t="str">
         <f aca="false">IF(N(D37)=0,"",Assumptions!$C$7/D37)</f>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C39" s="12" t="n">
         <f aca="false">Assumptions!$C$12</f>
-        <v>15.7142857142857</v>
+        <v>17.1428571428571</v>
       </c>
       <c r="D39" s="12" t="str">
         <f aca="false">IF(D37="","",Assumptions!$C$12)</f>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="C40" s="13" t="n">
         <f aca="false">IF(C39="","",C39-C37)</f>
-        <v>-0.0357142857142865</v>
+        <v>1.39285714285714</v>
       </c>
       <c r="D40" s="13" t="str">
         <f aca="false">IF(OR(D37="",D39=""),"",D39-D37)</f>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="C42" s="23" t="str">
         <f aca="false">IF(C38="","",IF(C38&gt;=Assumptions!$C$6,"Yes","No"))</f>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="D42" s="23" t="str">
         <f aca="false">IF(D38="","",IF(D38&gt;=Assumptions!$C$6,"Yes","No"))</f>

</xml_diff>